<commit_message>
code working some what
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/UPDATED TIMETABLE TOTAL.xlsx
+++ b/TIME TABLE SAMPLE DATA/UPDATED TIMETABLE TOTAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ganig\Desktop\Time_Table_\TIME TABLE SAMPLE DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\OneDrive\Desktop\Timetable\TIME TABLE SAMPLE DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2918608-FAE1-48A9-97E2-3325D22D4987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F7FE1-F0AD-4AE2-A892-095831FE1093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7CA5131F-FD47-46FE-8D38-CE3A574D862A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CA5131F-FD47-46FE-8D38-CE3A574D862A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -469,44 +469,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F52D849-8006-48A0-8D6B-88427B4C70FA}">
   <dimension ref="A1:AI29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" customWidth="1"/>
-    <col min="5" max="5" width="22.36328125" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" customWidth="1"/>
-    <col min="8" max="8" width="19.1796875" customWidth="1"/>
-    <col min="9" max="9" width="15.1796875" customWidth="1"/>
-    <col min="10" max="10" width="12.08984375" customWidth="1"/>
-    <col min="11" max="11" width="19.1796875" customWidth="1"/>
-    <col min="12" max="12" width="14.1796875" customWidth="1"/>
-    <col min="13" max="13" width="10.90625" customWidth="1"/>
-    <col min="14" max="14" width="19.1796875" customWidth="1"/>
-    <col min="15" max="15" width="12.54296875" customWidth="1"/>
-    <col min="16" max="16" width="10.90625" customWidth="1"/>
-    <col min="17" max="17" width="18.81640625" customWidth="1"/>
-    <col min="18" max="18" width="12.6328125" customWidth="1"/>
-    <col min="19" max="19" width="10.6328125" customWidth="1"/>
-    <col min="20" max="20" width="18.90625" customWidth="1"/>
-    <col min="21" max="21" width="12.6328125" customWidth="1"/>
-    <col min="22" max="22" width="10.54296875" customWidth="1"/>
-    <col min="23" max="23" width="17.90625" customWidth="1"/>
-    <col min="24" max="24" width="12.453125" customWidth="1"/>
-    <col min="25" max="25" width="11.90625" customWidth="1"/>
-    <col min="26" max="26" width="18.453125" customWidth="1"/>
-    <col min="27" max="27" width="13.08984375" customWidth="1"/>
-    <col min="28" max="28" width="11.08984375" customWidth="1"/>
-    <col min="29" max="29" width="18.08984375" customWidth="1"/>
-    <col min="30" max="30" width="12.90625" customWidth="1"/>
-    <col min="31" max="31" width="10.81640625" customWidth="1"/>
-    <col min="32" max="32" width="18.453125" customWidth="1"/>
-    <col min="33" max="33" width="13.54296875" customWidth="1"/>
-    <col min="34" max="34" width="10.90625" customWidth="1"/>
-    <col min="35" max="35" width="18.54296875" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" customWidth="1"/>
+    <col min="7" max="7" width="12.5546875" customWidth="1"/>
+    <col min="8" max="8" width="19.21875" customWidth="1"/>
+    <col min="9" max="9" width="15.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" customWidth="1"/>
+    <col min="11" max="11" width="19.21875" customWidth="1"/>
+    <col min="12" max="12" width="14.21875" customWidth="1"/>
+    <col min="13" max="13" width="10.88671875" customWidth="1"/>
+    <col min="14" max="14" width="19.21875" customWidth="1"/>
+    <col min="15" max="15" width="12.5546875" customWidth="1"/>
+    <col min="16" max="16" width="10.88671875" customWidth="1"/>
+    <col min="17" max="17" width="18.77734375" customWidth="1"/>
+    <col min="18" max="18" width="12.6640625" customWidth="1"/>
+    <col min="19" max="19" width="10.6640625" customWidth="1"/>
+    <col min="20" max="20" width="18.88671875" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" customWidth="1"/>
+    <col min="22" max="22" width="10.5546875" customWidth="1"/>
+    <col min="23" max="23" width="17.88671875" customWidth="1"/>
+    <col min="24" max="24" width="12.44140625" customWidth="1"/>
+    <col min="25" max="25" width="11.88671875" customWidth="1"/>
+    <col min="26" max="26" width="18.44140625" customWidth="1"/>
+    <col min="27" max="27" width="13.109375" customWidth="1"/>
+    <col min="28" max="28" width="11.109375" customWidth="1"/>
+    <col min="29" max="29" width="18.109375" customWidth="1"/>
+    <col min="30" max="30" width="12.88671875" customWidth="1"/>
+    <col min="31" max="31" width="10.77734375" customWidth="1"/>
+    <col min="32" max="32" width="18.44140625" customWidth="1"/>
+    <col min="33" max="33" width="13.5546875" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" customWidth="1"/>
+    <col min="35" max="35" width="18.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -569,7 +569,7 @@
       <c r="AH1" s="2"/>
       <c r="AI1" s="2"/>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" t="s">
@@ -672,7 +672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -779,7 +779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -886,7 +886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -993,7 +993,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>0</v>
       </c>
@@ -1880,7 +1880,7 @@
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" t="s">
@@ -1947,7 +1947,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3</v>
       </c>
@@ -2018,7 +2018,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>3</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>3</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>3</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>3</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>3</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>3</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>3</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>2</v>
       </c>
       <c r="G29">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H29">
         <v>2</v>
@@ -2680,7 +2680,7 @@
         <v>2</v>
       </c>
       <c r="J29">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K29">
         <v>2</v>
@@ -2724,6 +2724,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="AA1:AC1"/>
+    <mergeCell ref="AD1:AF1"/>
+    <mergeCell ref="AG1:AI1"/>
+    <mergeCell ref="U17:W17"/>
+    <mergeCell ref="U1:W1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="A17:A18"/>
@@ -2740,12 +2746,6 @@
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="AA1:AC1"/>
-    <mergeCell ref="AD1:AF1"/>
-    <mergeCell ref="AG1:AI1"/>
-    <mergeCell ref="U17:W17"/>
-    <mergeCell ref="U1:W1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>